<commit_message>
Marketing: 50-restaurant prospect list, loaded into the tracker's CRM
prospects.csv/.md: a research list of 50 Lahore restaurants, cafés and
dessert places fitting the ICP (16 A, 15 B, 19 C), each with a source
URL; handles and follower counts only where a source stated them. Not
contacted; every row needs verifying first. The tracker's CRM tab now
starts with these as 'To contact', sorted by priority.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aKz6B7AfHR6aSGKK8FgPS
</commit_message>
<xml_diff>
--- a/social/marketing/menva-marketing-tracker.xlsx
+++ b/social/marketing/menva-marketing-tracker.xlsx
@@ -5761,9 +5761,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>RARE Steakhouse</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd, Gulberg (rooftop, Gulberg Galleria)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium grill</t>
+        </is>
+      </c>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="6" t="n"/>
@@ -5772,13 +5784,25 @@
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="5" t="n"/>
-      <c r="L3" s="6" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M3" s="6" t="n"/>
       <c r="N3" s="5" t="n"/>
-      <c r="O3" s="6" t="n"/>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>Wagyu-focused steakhouse per source; premium cuts are exactly the 'how big is the cut' moment AR answers.</t>
+        </is>
+      </c>
       <c r="P3" s="5" t="n"/>
       <c r="Q3" s="6" t="n"/>
-      <c r="R3" s="6" t="n"/>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S3" s="5" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
@@ -5791,9 +5815,21 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Cafe Zouk</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd, Gulberg</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / steakhouse</t>
+        </is>
+      </c>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
@@ -5802,13 +5838,25 @@
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="5" t="n"/>
-      <c r="L4" s="6" t="n"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M4" s="6" t="n"/>
       <c r="N4" s="5" t="n"/>
-      <c r="O4" s="6" t="n"/>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>Sits in both the steakhouse and fine-dining source lists (ribeye/fillet/lamb steaks, Continental-Pan Asian-seafood menu) — dramatic plates, established brand.</t>
+        </is>
+      </c>
       <c r="P4" s="5" t="n"/>
       <c r="Q4" s="6" t="n"/>
-      <c r="R4" s="6" t="n"/>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S4" s="5" t="n"/>
       <c r="U4" s="2" t="inlineStr">
         <is>
@@ -5821,9 +5869,21 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Salt'n Pepper</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd, Gulberg (flagship)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium grill</t>
+        </is>
+      </c>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
@@ -5832,13 +5892,25 @@
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="6" t="n"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M5" s="6" t="n"/>
       <c r="N5" s="5" t="n"/>
-      <c r="O5" s="6" t="n"/>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Long-standing charcoal-grill brand on MM Alam Rd — established following, visually strong grilled plates.</t>
+        </is>
+      </c>
       <c r="P5" s="5" t="n"/>
       <c r="Q5" s="6" t="n"/>
-      <c r="R5" s="6" t="n"/>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S5" s="5" t="n"/>
       <c r="U5" s="2" t="inlineStr">
         <is>
@@ -5851,9 +5923,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Gaia</t>
+        </is>
+      </c>
       <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / Pan-Asian</t>
+        </is>
+      </c>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
@@ -5862,13 +5942,25 @@
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="5" t="n"/>
-      <c r="L6" s="6" t="n"/>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M6" s="6" t="n"/>
       <c r="N6" s="5" t="n"/>
-      <c r="O6" s="6" t="n"/>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>Described as premium Pan-Asian with theatrical teppanyaki grills and dark, moody luxury interior — a hero-dish moment AR can extend to the table.</t>
+        </is>
+      </c>
       <c r="P6" s="5" t="n"/>
       <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="6" t="n"/>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S6" s="5" t="n"/>
       <c r="U6" s="2" t="inlineStr">
         <is>
@@ -5881,9 +5973,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>The Skye</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg III (18th floor, Indigo Hotel)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / rooftop</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
@@ -5892,13 +5996,25 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M7" s="6" t="n"/>
       <c r="N7" s="5" t="n"/>
-      <c r="O7" s="6" t="n"/>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>Billed as Lahore's highest rooftop dining destination with 360-degree skyline views — premium experience spend, owner likely to see AR as the same category.</t>
+        </is>
+      </c>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="6" t="n"/>
-      <c r="R7" s="6" t="n"/>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S7" s="5" t="n"/>
       <c r="U7" s="2" t="inlineStr">
         <is>
@@ -5911,9 +6027,21 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>El Momento Steakhouse</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd, Gulberg 2</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium grill</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
@@ -5922,13 +6050,25 @@
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="5" t="n"/>
-      <c r="L8" s="6" t="n"/>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M8" s="6" t="n"/>
       <c r="N8" s="5" t="n"/>
-      <c r="O8" s="6" t="n"/>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>Tops multiple 2026 steakhouse rankings; imported aged beef cuts, sophisticated ambiance — same category as the pilot dish (steak board).</t>
+        </is>
+      </c>
       <c r="P8" s="5" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="6" t="n"/>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S8" s="5" t="n"/>
       <c r="U8" s="2" t="inlineStr">
         <is>
@@ -5941,9 +6081,21 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Cafe Aylanto</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / Mediterranean</t>
+        </is>
+      </c>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
@@ -5952,13 +6104,25 @@
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="5" t="n"/>
-      <c r="L9" s="6" t="n"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M9" s="6" t="n"/>
       <c r="N9" s="5" t="n"/>
-      <c r="O9" s="6" t="n"/>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>Long-running benchmark for upscale Mediterranean dining in Lahore — brand-conscious owner likely to value a tasteful AR menu over a gimmick.</t>
+        </is>
+      </c>
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="6" t="n"/>
-      <c r="R9" s="6" t="n"/>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S9" s="5" t="n"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
@@ -5971,9 +6135,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n"/>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Sikomoro</t>
+        </is>
+      </c>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / new opening</t>
+        </is>
+      </c>
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
@@ -5982,13 +6154,25 @@
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="5" t="n"/>
-      <c r="L10" s="6" t="n"/>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M10" s="6" t="n"/>
       <c r="N10" s="5" t="n"/>
-      <c r="O10" s="6" t="n"/>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>New poolside dining spot with French/Italian/continental plates and an in-house bakery — pre-launch or early menu means no legacy PDF to fight.</t>
+        </is>
+      </c>
       <c r="P10" s="5" t="n"/>
       <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="n"/>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S10" s="5" t="n"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
@@ -6001,9 +6185,21 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Olive Fork</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town Lahore (opposite Grand Masjid)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>New opening</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
@@ -6012,19 +6208,43 @@
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="5" t="n"/>
-      <c r="L11" s="6" t="n"/>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="5" t="n"/>
-      <c r="O11" s="6" t="n"/>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>Recently opened per source — early-days restaurants are the easiest 'yes' before their menu is printed.</t>
+        </is>
+      </c>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="6" t="n"/>
-      <c r="R11" s="6" t="n"/>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Andaaz</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Fort Road, near Badshahi Mosque</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / heritage rooftop</t>
+        </is>
+      </c>
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
@@ -6033,19 +6253,43 @@
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="5" t="n"/>
-      <c r="L12" s="6" t="n"/>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M12" s="6" t="n"/>
       <c r="N12" s="5" t="n"/>
-      <c r="O12" s="6" t="n"/>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>Rooftop Pakistani fine dining combining heritage setting with plated food — visually strong, tourist and status-dining crowd.</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="6" t="n"/>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Arizona Grill</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / grill</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
@@ -6054,19 +6298,39 @@
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="5" t="n"/>
-      <c r="L13" s="6" t="n"/>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M13" s="6" t="n"/>
       <c r="N13" s="5" t="n"/>
-      <c r="O13" s="6" t="n"/>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>Steaks, burgers and grilled sandwiches in a newer commercial area with less marketing-tech saturation, per sales-kit area logic.</t>
+        </is>
+      </c>
       <c r="P13" s="5" t="n"/>
       <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="n"/>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Spice Bazaar</t>
+        </is>
+      </c>
       <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / Pakistani</t>
+        </is>
+      </c>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
@@ -6075,19 +6339,43 @@
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="5" t="n"/>
-      <c r="L14" s="6" t="n"/>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M14" s="6" t="n"/>
       <c r="N14" s="5" t="n"/>
-      <c r="O14" s="6" t="n"/>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>Established Pakistani fine-dining name (has its own Wikipedia page) — status-dining crowd, plated hero dishes.</t>
+        </is>
+      </c>
       <c r="P14" s="5" t="n"/>
       <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="6" t="n"/>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok Steakhouse</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium grill</t>
+        </is>
+      </c>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
@@ -6096,19 +6384,43 @@
       <c r="I15" s="5" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="5" t="n"/>
-      <c r="L15" s="6" t="n"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M15" s="6" t="n"/>
       <c r="N15" s="5" t="n"/>
-      <c r="O15" s="6" t="n"/>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>Local favourite for generous grilled portions and marinades — the portion-size question AR is built to answer.</t>
+        </is>
+      </c>
       <c r="P15" s="5" t="n"/>
       <c r="Q15" s="6" t="n"/>
-      <c r="R15" s="6" t="n"/>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Xander's</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>MM Alam Rd, Gulberg</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium casual grill</t>
+        </is>
+      </c>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
@@ -6117,19 +6429,39 @@
       <c r="I16" s="5" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="5" t="n"/>
-      <c r="L16" s="6" t="n"/>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M16" s="6" t="n"/>
       <c r="N16" s="5" t="n"/>
-      <c r="O16" s="6" t="n"/>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>Casual-upscale steaks and grilled meats on MM Alam Rd — fits premium casual grill category directly.</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="n"/>
       <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="6" t="n"/>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Promenade</t>
+        </is>
+      </c>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / new opening</t>
+        </is>
+      </c>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
@@ -6138,19 +6470,39 @@
       <c r="I17" s="5" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="5" t="n"/>
-      <c r="L17" s="6" t="n"/>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M17" s="6" t="n"/>
       <c r="N17" s="5" t="n"/>
-      <c r="O17" s="6" t="n"/>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>Reported as Pakistan's first Bridgerton-themed cafe in Lahore — high novelty and photo appeal, natural fit for an AR menu as a launch story.</t>
+        </is>
+      </c>
       <c r="P17" s="5" t="n"/>
       <c r="Q17" s="6" t="n"/>
-      <c r="R17" s="6" t="n"/>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n"/>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Mystique Restaurant</t>
+        </is>
+      </c>
       <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining</t>
+        </is>
+      </c>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
@@ -6159,19 +6511,39 @@
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="5" t="n"/>
-      <c r="L18" s="6" t="n"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M18" s="6" t="n"/>
       <c r="N18" s="5" t="n"/>
-      <c r="O18" s="6" t="n"/>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>Self-described upscale spot blending continental, Asian and Pakistani dishes, positioned for corporate dinners and special occasions — experience-spend owner.</t>
+        </is>
+      </c>
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="6" t="n"/>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority A), then first contact</t>
+        </is>
+      </c>
       <c r="S18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Dahlia Nursery + Cafe</t>
+        </is>
+      </c>
       <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe</t>
+        </is>
+      </c>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
@@ -6180,19 +6552,39 @@
       <c r="I19" s="5" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="5" t="n"/>
-      <c r="L19" s="6" t="n"/>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M19" s="6" t="n"/>
       <c r="N19" s="5" t="n"/>
-      <c r="O19" s="6" t="n"/>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>Plant-filled nursery-cafe aesthetic — guests already photograph the space; natural extension to photograph/AR the dish too.</t>
+        </is>
+      </c>
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="6" t="n"/>
-      <c r="R19" s="6" t="n"/>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n"/>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Cafe Forest 14</t>
+        </is>
+      </c>
       <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe</t>
+        </is>
+      </c>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
@@ -6201,19 +6593,39 @@
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="5" t="n"/>
-      <c r="L20" s="6" t="n"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M20" s="6" t="n"/>
       <c r="N20" s="5" t="n"/>
-      <c r="O20" s="6" t="n"/>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>"Bali in Lahore" indoor-forest theme built for sunset photography — strong Instagram-first crowd.</t>
+        </is>
+      </c>
       <c r="P20" s="5" t="n"/>
       <c r="Q20" s="6" t="n"/>
-      <c r="R20" s="6" t="n"/>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Bistro Noir</t>
+        </is>
+      </c>
       <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe</t>
+        </is>
+      </c>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
@@ -6222,19 +6634,39 @@
       <c r="I21" s="5" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="5" t="n"/>
-      <c r="L21" s="6" t="n"/>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M21" s="6" t="n"/>
       <c r="N21" s="5" t="n"/>
-      <c r="O21" s="6" t="n"/>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>Monochrome, minimalist-luxury styling described as a deliberate design statement — brand-conscious owner.</t>
+        </is>
+      </c>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="6" t="n"/>
-      <c r="R21" s="6" t="n"/>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n"/>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Yanu</t>
+        </is>
+      </c>
       <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / poolside</t>
+        </is>
+      </c>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
@@ -6243,19 +6675,39 @@
       <c r="I22" s="5" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="5" t="n"/>
-      <c r="L22" s="6" t="n"/>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M22" s="6" t="n"/>
       <c r="N22" s="5" t="n"/>
-      <c r="O22" s="6" t="n"/>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>Described as a Pinterest-style poolside spot for brunch and evening photoshoots — guests are already in a photograph-the-food mindset.</t>
+        </is>
+      </c>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="6" t="n"/>
-      <c r="R22" s="6" t="n"/>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n"/>
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Meet Me In Paris</t>
+        </is>
+      </c>
       <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe</t>
+        </is>
+      </c>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
@@ -6264,19 +6716,39 @@
       <c r="I23" s="5" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="5" t="n"/>
-      <c r="L23" s="6" t="n"/>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M23" s="6" t="n"/>
       <c r="N23" s="5" t="n"/>
-      <c r="O23" s="6" t="n"/>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>Floral facade described as one of the most photographed cafe entrances in Lahore — proof guests already stop to photograph before they order.</t>
+        </is>
+      </c>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="6" t="n"/>
-      <c r="R23" s="6" t="n"/>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n"/>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>COMO Museum of Art Cafe</t>
+        </is>
+      </c>
       <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / gallery</t>
+        </is>
+      </c>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
@@ -6285,19 +6757,39 @@
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="5" t="n"/>
-      <c r="L24" s="6" t="n"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M24" s="6" t="n"/>
       <c r="N24" s="5" t="n"/>
-      <c r="O24" s="6" t="n"/>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>Cafe inside an art museum, modern architecture — audience already primed for a considered visual experience.</t>
+        </is>
+      </c>
       <c r="P24" s="5" t="n"/>
       <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="6" t="n"/>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n"/>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Deja by Khadija</t>
+        </is>
+      </c>
       <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic dessert cafe</t>
+        </is>
+      </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
@@ -6306,19 +6798,43 @@
       <c r="I25" s="5" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="5" t="n"/>
-      <c r="L25" s="6" t="n"/>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M25" s="6" t="n"/>
       <c r="N25" s="5" t="n"/>
-      <c r="O25" s="6" t="n"/>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>Pink-and-white dessert cafe described as "every corner is picture-perfect" — decorated cakes are a hero-dish candidate.</t>
+        </is>
+      </c>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="6" t="n"/>
-      <c r="R25" s="6" t="n"/>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Sweet Affairs</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg + DHA</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / dessert</t>
+        </is>
+      </c>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="n"/>
@@ -6327,19 +6843,43 @@
       <c r="I26" s="5" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="5" t="n"/>
-      <c r="L26" s="6" t="n"/>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M26" s="6" t="n"/>
       <c r="N26" s="5" t="n"/>
-      <c r="O26" s="6" t="n"/>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>Whimsical, pastel decor since 2011; skillet-cookie dessert is a shareable, photogenic hero item.</t>
+        </is>
+      </c>
       <c r="P26" s="5" t="n"/>
       <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="6" t="n"/>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>The Urban Eatery</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>DHA</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / casual dining</t>
+        </is>
+      </c>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
@@ -6348,19 +6888,43 @@
       <c r="I27" s="5" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="5" t="n"/>
-      <c r="L27" s="6" t="n"/>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M27" s="6" t="n"/>
       <c r="N27" s="5" t="n"/>
-      <c r="O27" s="6" t="n"/>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>Listed among Lahore's aesthetic hangout spots — established Instagram-forward brunch crowd.</t>
+        </is>
+      </c>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="6" t="n"/>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>English Tea House</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg + DHA</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Photogenic cafe / breakfast</t>
+        </is>
+      </c>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
@@ -6369,19 +6933,43 @@
       <c r="I28" s="5" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="5" t="n"/>
-      <c r="L28" s="6" t="n"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M28" s="6" t="n"/>
       <c r="N28" s="5" t="n"/>
-      <c r="O28" s="6" t="n"/>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>Listed among Lahore's aesthetic hangout spots for breakfast — photogenic plating, brunch crowd.</t>
+        </is>
+      </c>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="6" t="n"/>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Sweet Tooth</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Mall 1</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Dessert cafe</t>
+        </is>
+      </c>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
@@ -6390,19 +6978,39 @@
       <c r="I29" s="5" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="5" t="n"/>
-      <c r="L29" s="6" t="n"/>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M29" s="6" t="n"/>
       <c r="N29" s="5" t="n"/>
-      <c r="O29" s="6" t="n"/>
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>Described as one of the newest Instagrammable dessert spots in town, with wall art and a cozy setting built for photos.</t>
+        </is>
+      </c>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="6" t="n"/>
+      <c r="R29" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n"/>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Layers - Bakeshop</t>
+        </is>
+      </c>
       <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Dessert / bakery</t>
+        </is>
+      </c>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
@@ -6411,19 +7019,39 @@
       <c r="I30" s="5" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="5" t="n"/>
-      <c r="L30" s="6" t="n"/>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M30" s="6" t="n"/>
       <c r="N30" s="5" t="n"/>
-      <c r="O30" s="6" t="n"/>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>Affordable cupcakes, cakes and sundaes (Galaxy Sundae, salted caramel cake called out by name) — visual, shareable desserts.</t>
+        </is>
+      </c>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="6" t="n"/>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Dessert Directory</t>
+        </is>
+      </c>
       <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Dessert / boutique bakery</t>
+        </is>
+      </c>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
@@ -6432,19 +7060,43 @@
       <c r="I31" s="5" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="5" t="n"/>
-      <c r="L31" s="6" t="n"/>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M31" s="6" t="n"/>
       <c r="N31" s="5" t="n"/>
-      <c r="O31" s="6" t="n"/>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>French-inspired boutique dessert shop aggregating home-based bakers — novelty, photogenic packaging.</t>
+        </is>
+      </c>
       <c r="P31" s="5" t="n"/>
       <c r="Q31" s="6" t="n"/>
-      <c r="R31" s="6" t="n"/>
+      <c r="R31" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Freddy's Cafe</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Premium casual / continental</t>
+        </is>
+      </c>
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
@@ -6453,19 +7105,43 @@
       <c r="I32" s="5" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="5" t="n"/>
-      <c r="L32" s="6" t="n"/>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M32" s="6" t="n"/>
       <c r="N32" s="5" t="n"/>
-      <c r="O32" s="6" t="n"/>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>Stylish continental dining known for pastas and steaks — premium casual fit outside the Gulberg/DHA cluster.</t>
+        </is>
+      </c>
       <c r="P32" s="5" t="n"/>
       <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="6" t="n"/>
+      <c r="R32" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>FiLLi Cafe</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town (and other Lahore branches)</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Cafe / tea chain</t>
+        </is>
+      </c>
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
@@ -6474,19 +7150,43 @@
       <c r="I33" s="5" t="n"/>
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="5" t="n"/>
-      <c r="L33" s="6" t="n"/>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M33" s="6" t="n"/>
       <c r="N33" s="5" t="n"/>
-      <c r="O33" s="6" t="n"/>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>Known for a signature Zafran Chai and a strong local following — large audience, worth checking whether the printed menu is text-only.</t>
+        </is>
+      </c>
       <c r="P33" s="5" t="n"/>
       <c r="Q33" s="6" t="n"/>
-      <c r="R33" s="6" t="n"/>
+      <c r="R33" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority B), then first contact</t>
+        </is>
+      </c>
       <c r="S33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Howdy</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / premium casual</t>
+        </is>
+      </c>
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
@@ -6495,19 +7195,43 @@
       <c r="I34" s="5" t="n"/>
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="5" t="n"/>
-      <c r="L34" s="6" t="n"/>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M34" s="6" t="n"/>
       <c r="N34" s="5" t="n"/>
-      <c r="O34" s="6" t="n"/>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>Described as a premium, cowboy-themed steakhouse for burgers and steaks — verify it is not primarily a fast-food/burger operation before pitching.</t>
+        </is>
+      </c>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="6" t="n"/>
-      <c r="R34" s="6" t="n"/>
+      <c r="R34" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Ranchers</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Steakhouse / grill</t>
+        </is>
+      </c>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
@@ -6516,19 +7240,43 @@
       <c r="I35" s="5" t="n"/>
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="5" t="n"/>
-      <c r="L35" s="6" t="n"/>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M35" s="6" t="n"/>
       <c r="N35" s="5" t="n"/>
-      <c r="O35" s="6" t="n"/>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>Described as a meat-lovers spot for grilled steaks in a rustic setting.</t>
+        </is>
+      </c>
       <c r="P35" s="5" t="n"/>
       <c r="Q35" s="6" t="n"/>
-      <c r="R35" s="6" t="n"/>
+      <c r="R35" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Double Shot Coffee</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>DHA Phase 6</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Cafe / coffee</t>
+        </is>
+      </c>
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="n"/>
@@ -6537,19 +7285,43 @@
       <c r="I36" s="5" t="n"/>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="5" t="n"/>
-      <c r="L36" s="6" t="n"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M36" s="6" t="n"/>
       <c r="N36" s="5" t="n"/>
-      <c r="O36" s="6" t="n"/>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>Coffee-forward modern cafe in the DHA Phase 6 cluster — good for a single-afternoon walk with other DHA prospects.</t>
+        </is>
+      </c>
       <c r="P36" s="5" t="n"/>
       <c r="Q36" s="6" t="n"/>
-      <c r="R36" s="6" t="n"/>
+      <c r="R36" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Kickstart Cafe</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>DHA Phase 6</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Cafe</t>
+        </is>
+      </c>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
@@ -6558,19 +7330,43 @@
       <c r="I37" s="5" t="n"/>
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="5" t="n"/>
-      <c r="L37" s="6" t="n"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M37" s="6" t="n"/>
       <c r="N37" s="5" t="n"/>
-      <c r="O37" s="6" t="n"/>
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>Positively reviewed neighbourhood cafe in the DHA Phase 6 cluster.</t>
+        </is>
+      </c>
       <c r="P37" s="5" t="n"/>
       <c r="Q37" s="6" t="n"/>
-      <c r="R37" s="6" t="n"/>
+      <c r="R37" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Chai Hujra</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>DHA Phase 5</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Cafe / evening venue</t>
+        </is>
+      </c>
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="6" t="n"/>
@@ -6579,19 +7375,43 @@
       <c r="I38" s="5" t="n"/>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="5" t="n"/>
-      <c r="L38" s="6" t="n"/>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M38" s="6" t="n"/>
       <c r="N38" s="5" t="n"/>
-      <c r="O38" s="6" t="n"/>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>Nightly live-music tea venue in DHA Phase 5 — verify it has a plated food menu (not just tea/snacks) before treating as an AR-menu fit.</t>
+        </is>
+      </c>
       <c r="P38" s="5" t="n"/>
       <c r="Q38" s="6" t="n"/>
-      <c r="R38" s="6" t="n"/>
+      <c r="R38" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Kudo's Caff</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Cafe</t>
+        </is>
+      </c>
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
@@ -6600,19 +7420,43 @@
       <c r="I39" s="5" t="n"/>
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="5" t="n"/>
-      <c r="L39" s="6" t="n"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M39" s="6" t="n"/>
       <c r="N39" s="5" t="n"/>
-      <c r="O39" s="6" t="n"/>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>Trendy neighbourhood cafe for casual meetups and coffee.</t>
+        </is>
+      </c>
       <c r="P39" s="5" t="n"/>
       <c r="Q39" s="6" t="n"/>
-      <c r="R39" s="6" t="n"/>
+      <c r="R39" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Buqayvia Restaurant</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Casual dining / Pakistani-continental</t>
+        </is>
+      </c>
       <c r="D40" s="6" t="n"/>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="6" t="n"/>
@@ -6621,19 +7465,43 @@
       <c r="I40" s="5" t="n"/>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="5" t="n"/>
-      <c r="L40" s="6" t="n"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M40" s="6" t="n"/>
       <c r="N40" s="5" t="n"/>
-      <c r="O40" s="6" t="n"/>
+      <c r="O40" s="6" t="inlineStr">
+        <is>
+          <t>Family-casual Pakistani/continental spot — screen for table service and a hero dish before pitching.</t>
+        </is>
+      </c>
       <c r="P40" s="5" t="n"/>
       <c r="Q40" s="6" t="n"/>
-      <c r="R40" s="6" t="n"/>
+      <c r="R40" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Chaye Qawali</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Cafe / tea</t>
+        </is>
+      </c>
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
@@ -6642,19 +7510,43 @@
       <c r="I41" s="5" t="n"/>
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="5" t="n"/>
-      <c r="L41" s="6" t="n"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M41" s="6" t="n"/>
       <c r="N41" s="5" t="n"/>
-      <c r="O41" s="6" t="n"/>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>Tea-focused cafe with a vibrant atmosphere — check whether food menu has a strong-enough hero dish for AR.</t>
+        </is>
+      </c>
       <c r="P41" s="5" t="n"/>
       <c r="Q41" s="6" t="n"/>
-      <c r="R41" s="6" t="n"/>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="6" t="n"/>
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Al-Nakhal Arabian Cuisine</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Johar Town</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Restaurant / Arabian</t>
+        </is>
+      </c>
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
@@ -6663,19 +7555,43 @@
       <c r="I42" s="5" t="n"/>
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="5" t="n"/>
-      <c r="L42" s="6" t="n"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M42" s="6" t="n"/>
       <c r="N42" s="5" t="n"/>
-      <c r="O42" s="6" t="n"/>
+      <c r="O42" s="6" t="inlineStr">
+        <is>
+          <t>Arabian cuisine (mandi/platter-style dishes tend to be visually dramatic and shareable) — worth a screen visit.</t>
+        </is>
+      </c>
       <c r="P42" s="5" t="n"/>
       <c r="Q42" s="6" t="n"/>
-      <c r="R42" s="6" t="n"/>
+      <c r="R42" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="6" t="n"/>
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>The Lost Tribe</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Model Town</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Casual dining / Pakistani</t>
+        </is>
+      </c>
       <c r="D43" s="6" t="n"/>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
@@ -6684,19 +7600,43 @@
       <c r="I43" s="5" t="n"/>
       <c r="J43" s="6" t="n"/>
       <c r="K43" s="5" t="n"/>
-      <c r="L43" s="6" t="n"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M43" s="6" t="n"/>
       <c r="N43" s="5" t="n"/>
-      <c r="O43" s="6" t="n"/>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>Described as blending tradition with modern culinary presentation — Model Town referral cluster per sales-kit area logic.</t>
+        </is>
+      </c>
       <c r="P43" s="5" t="n"/>
       <c r="Q43" s="6" t="n"/>
-      <c r="R43" s="6" t="n"/>
+      <c r="R43" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Model Town Club</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Model Town</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Restaurant / club dining</t>
+        </is>
+      </c>
       <c r="D44" s="6" t="n"/>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="6" t="n"/>
@@ -6705,19 +7645,43 @@
       <c r="I44" s="5" t="n"/>
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="5" t="n"/>
-      <c r="L44" s="6" t="n"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M44" s="6" t="n"/>
       <c r="N44" s="5" t="n"/>
-      <c r="O44" s="6" t="n"/>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>BBQ, kebabs and an international menu inside a members' club — check decision-maker access (club vs. owner-operator) before pitching.</t>
+        </is>
+      </c>
       <c r="P44" s="5" t="n"/>
       <c r="Q44" s="6" t="n"/>
-      <c r="R44" s="6" t="n"/>
+      <c r="R44" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="6" t="n"/>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Cafe Grand</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town (Sector B, Bahria Grand Hotel)</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / gourmet casual</t>
+        </is>
+      </c>
       <c r="D45" s="6" t="n"/>
       <c r="E45" s="6" t="n"/>
       <c r="F45" s="6" t="n"/>
@@ -6726,19 +7690,43 @@
       <c r="I45" s="5" t="n"/>
       <c r="J45" s="6" t="n"/>
       <c r="K45" s="5" t="n"/>
-      <c r="L45" s="6" t="n"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M45" s="6" t="n"/>
       <c r="N45" s="5" t="n"/>
-      <c r="O45" s="6" t="n"/>
+      <c r="O45" s="6" t="inlineStr">
+        <is>
+          <t>Called the best casual-gourmet spot in Bahria Town in one source — hotel-based, so confirm who actually decides on a paid pilot.</t>
+        </is>
+      </c>
       <c r="P45" s="5" t="n"/>
       <c r="Q45" s="6" t="n"/>
-      <c r="R45" s="6" t="n"/>
+      <c r="R45" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Mei Kong</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town (Sector C Commercial)</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / Chinese-Asian</t>
+        </is>
+      </c>
       <c r="D46" s="6" t="n"/>
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="6" t="n"/>
@@ -6747,19 +7735,43 @@
       <c r="I46" s="5" t="n"/>
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="5" t="n"/>
-      <c r="L46" s="6" t="n"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M46" s="6" t="n"/>
       <c r="N46" s="5" t="n"/>
-      <c r="O46" s="6" t="n"/>
+      <c r="O46" s="6" t="inlineStr">
+        <is>
+          <t>Described as upscale Chinese/Asian dining — newer commercial area, less marketing-tech saturation.</t>
+        </is>
+      </c>
       <c r="P46" s="5" t="n"/>
       <c r="Q46" s="6" t="n"/>
-      <c r="R46" s="6" t="n"/>
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>The Monal</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Rooftop / multi-cuisine</t>
+        </is>
+      </c>
       <c r="D47" s="6" t="n"/>
       <c r="E47" s="6" t="n"/>
       <c r="F47" s="6" t="n"/>
@@ -6768,19 +7780,43 @@
       <c r="I47" s="5" t="n"/>
       <c r="J47" s="6" t="n"/>
       <c r="K47" s="5" t="n"/>
-      <c r="L47" s="6" t="n"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M47" s="6" t="n"/>
       <c r="N47" s="5" t="n"/>
-      <c r="O47" s="6" t="n"/>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>Rooftop view dining (Pakistani/Chinese/continental) — check for a hero dish worth an AR scan.</t>
+        </is>
+      </c>
       <c r="P47" s="5" t="n"/>
       <c r="Q47" s="6" t="n"/>
-      <c r="R47" s="6" t="n"/>
+      <c r="R47" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Ginsoy</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Bahria Town</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Fine dining / Chinese-Thai</t>
+        </is>
+      </c>
       <c r="D48" s="6" t="n"/>
       <c r="E48" s="6" t="n"/>
       <c r="F48" s="6" t="n"/>
@@ -6789,19 +7825,43 @@
       <c r="I48" s="5" t="n"/>
       <c r="J48" s="6" t="n"/>
       <c r="K48" s="5" t="n"/>
-      <c r="L48" s="6" t="n"/>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M48" s="6" t="n"/>
       <c r="N48" s="5" t="n"/>
-      <c r="O48" s="6" t="n"/>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>Asian cuisine spot called out as a strong option in Bahria Town.</t>
+        </is>
+      </c>
       <c r="P48" s="5" t="n"/>
       <c r="Q48" s="6" t="n"/>
-      <c r="R48" s="6" t="n"/>
+      <c r="R48" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="6" t="n"/>
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Waleed's Kitchen</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>PIA Road</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>New opening</t>
+        </is>
+      </c>
       <c r="D49" s="6" t="n"/>
       <c r="E49" s="6" t="n"/>
       <c r="F49" s="6" t="n"/>
@@ -6810,40 +7870,92 @@
       <c r="I49" s="5" t="n"/>
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="5" t="n"/>
-      <c r="L49" s="6" t="n"/>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M49" s="6" t="n"/>
       <c r="N49" s="5" t="n"/>
-      <c r="O49" s="6" t="n"/>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>Reported as a new food spot on PIA Road — category and hero dish unconfirmed, screen before pitching.</t>
+        </is>
+      </c>
       <c r="P49" s="5" t="n"/>
       <c r="Q49" s="6" t="n"/>
-      <c r="R49" s="6" t="n"/>
+      <c r="R49" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Chow Ming</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>DHA Phase 4, Bahria Town, Johar Town</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Casual dining / multi-branch</t>
+        </is>
+      </c>
       <c r="D50" s="6" t="n"/>
       <c r="E50" s="6" t="n"/>
       <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>chowmingpk</t>
+        </is>
+      </c>
       <c r="H50" s="6" t="n"/>
       <c r="I50" s="5" t="n"/>
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="5" t="n"/>
-      <c r="L50" s="6" t="n"/>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M50" s="6" t="n"/>
       <c r="N50" s="5" t="n"/>
-      <c r="O50" s="6" t="n"/>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>Multi-branch casual chain with an active Instagram presence — per screening criteria, multi-branch chains are a slower first-90-days approval, so treat as a later-stage lead.</t>
+        </is>
+      </c>
       <c r="P50" s="5" t="n"/>
       <c r="Q50" s="6" t="n"/>
-      <c r="R50" s="6" t="n"/>
+      <c r="R50" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="6" t="n"/>
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Meat The Cheese</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Casual dining / grill</t>
+        </is>
+      </c>
       <c r="D51" s="6" t="n"/>
       <c r="E51" s="6" t="n"/>
       <c r="F51" s="6" t="n"/>
@@ -6852,19 +7964,43 @@
       <c r="I51" s="5" t="n"/>
       <c r="J51" s="6" t="n"/>
       <c r="K51" s="5" t="n"/>
-      <c r="L51" s="6" t="n"/>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M51" s="6" t="n"/>
       <c r="N51" s="5" t="n"/>
-      <c r="O51" s="6" t="n"/>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>Listed among Gulberg's dine-in destinations — verify current hero dish and table-service format.</t>
+        </is>
+      </c>
       <c r="P51" s="5" t="n"/>
       <c r="Q51" s="6" t="n"/>
-      <c r="R51" s="6" t="n"/>
+      <c r="R51" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>The Brasserie</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Gulberg</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Casual dining</t>
+        </is>
+      </c>
       <c r="D52" s="6" t="n"/>
       <c r="E52" s="6" t="n"/>
       <c r="F52" s="6" t="n"/>
@@ -6873,13 +8009,25 @@
       <c r="I52" s="5" t="n"/>
       <c r="J52" s="6" t="n"/>
       <c r="K52" s="5" t="n"/>
-      <c r="L52" s="6" t="n"/>
+      <c r="L52" s="6" t="inlineStr">
+        <is>
+          <t>To contact</t>
+        </is>
+      </c>
       <c r="M52" s="6" t="n"/>
       <c r="N52" s="5" t="n"/>
-      <c r="O52" s="6" t="n"/>
+      <c r="O52" s="6" t="inlineStr">
+        <is>
+          <t>Listed among Gulberg's dine-in destinations — verify current concept and menu format.</t>
+        </is>
+      </c>
       <c r="P52" s="5" t="n"/>
       <c r="Q52" s="6" t="n"/>
-      <c r="R52" s="6" t="n"/>
+      <c r="R52" s="6" t="inlineStr">
+        <is>
+          <t>Verify it still fits (priority C), then first contact</t>
+        </is>
+      </c>
       <c r="S52" s="5" t="n"/>
     </row>
     <row r="53">

</xml_diff>

<commit_message>
Tracker: content log refreshed with the rewritten headlines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aKz6B7AfHR6aSGKK8FgPS
</commit_message>
<xml_diff>
--- a/social/marketing/menva-marketing-tracker.xlsx
+++ b/social/marketing/menva-marketing-tracker.xlsx
@@ -1680,7 +1680,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>The waiter is back. Again.</t>
+          <t>The waiter's back. Still on page two.</t>
         </is>
       </c>
       <c r="I3" s="6" t="n"/>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>This is a scan, not a photo.</t>
+          <t>Not a photo. A full 3D scan.</t>
         </is>
       </c>
       <c r="I4" s="6" t="n"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Friday night. Pick one.</t>
+          <t>Friday, 9 pm. Pick one.</t>
         </is>
       </c>
       <c r="I5" s="6" t="n"/>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Ordering for eight, without the chaos.</t>
+          <t>Group of eight. One order, not eight arguments.</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Your menu is your quietest salesperson.</t>
+          <t>Your menu sells before anyone speaks.</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Menu photos lie. Scans don't.</t>
+          <t>That photo's from 2019. The plate isn't.</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Scan the code on your table</t>
+          <t>Scan the code already on your table</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Order what you actually want.</t>
+          <t>Order what you actually wanted.</t>
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>You didn't check the portion size.</t>
+          <t>You ordered a starter. It arrived on a board.</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>New restaurant. New menu. Same order.</t>
+          <t>New menu. Same order. Every time.</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Turn it around.</t>
+          <t>Check the other side first.</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>The most asked question in your restaurant: "What does it look like?"</t>
+          <t>"What does this even look like?"</t>
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Weekend plans, sorted.</t>
+          <t>Where to go: 2 minutes. What to order: 45.</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Twelve pages. No pictures. The waiter is watching.</t>
+          <t>Twelve pages. No pictures. Waiter is watching.</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Your plating, before the order.</t>
+          <t>Years on plating. Eleven words on a page.</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Lunch or dinner, pick one.</t>
+          <t>One's on a plate, one's on a board.</t>
         </is>
       </c>
       <c r="I20" s="6" t="n"/>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>The scariest thing in Lahore tonight is a menu with no photos.</t>
+          <t>Scariest thing in Lahore tonight? A menu with zero photos.</t>
         </is>
       </c>
       <c r="I21" s="6" t="n"/>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Date night. No surprises.</t>
+          <t>Rule one: don't order the messiest thing.</t>
         </is>
       </c>
       <c r="I22" s="6" t="n"/>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Smog outside. Good food inside.</t>
+          <t>Outdoor plans just became indoor plans.</t>
         </is>
       </c>
       <c r="I23" s="6" t="n"/>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>No zoom. No tricks. True size.</t>
+          <t>You can't pinch it bigger.</t>
         </is>
       </c>
       <c r="I25" s="6" t="n"/>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Which one makes you hungry?</t>
+          <t>Which one makes you actually hungry?</t>
         </is>
       </c>
       <c r="I28" s="6" t="n"/>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>The over-orderer.</t>
+          <t>The over-orderer, itemised.</t>
         </is>
       </c>
       <c r="I30" s="6" t="n"/>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Five signs your menu is costing you orders</t>
+          <t>Five signs your menu's costing you orders</t>
         </is>
       </c>
       <c r="I32" s="6" t="n"/>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>No AI food. Ever.</t>
+          <t>No AI-generated food. Not once, not ever.</t>
         </is>
       </c>
       <c r="I34" s="6" t="n"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>"Is it worth the hype?" Decide before you order.</t>
+          <t>"Is it worth the hype?"</t>
         </is>
       </c>
       <c r="I35" s="6" t="n"/>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Shaadi ka khana fix hai.</t>
+          <t>Zero control over the menu.</t>
         </is>
       </c>
       <c r="I38" s="6" t="n"/>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Let the menu show the plate. Let your team host.</t>
+          <t>Let the menu do the describing. Let your team host.</t>
         </is>
       </c>
       <c r="I42" s="6" t="n"/>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>Cold nights. Long dinners.</t>
+          <t>Every friend's back in town.</t>
         </is>
       </c>
       <c r="I43" s="6" t="n"/>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>You pick the angle.</t>
+          <t>Above. Side. Underneath. Your choice.</t>
         </is>
       </c>
       <c r="I46" s="6" t="n"/>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>When their plate arrives and it looks better than yours.</t>
+          <t>Their plate always looks better.</t>
         </is>
       </c>
       <c r="I48" s="6" t="n"/>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Cold night. Pick one.</t>
+          <t>Cold night, one plate.</t>
         </is>
       </c>
       <c r="I49" s="6" t="n"/>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>The food critic.</t>
+          <t>The food critic</t>
         </is>
       </c>
       <c r="I51" s="6" t="n"/>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>Trying a new place? Checklist.</t>
+          <t>Checklist before you order</t>
         </is>
       </c>
       <c r="I56" s="6" t="n"/>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>Last dinner of the year. Make it count.</t>
+          <t>Last dinner. Make it count.</t>
         </is>
       </c>
       <c r="I64" s="6" t="n"/>

</xml_diff>

<commit_message>
Refreshed previews, profile grid and tracker after the spicier pass
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aKz6B7AfHR6aSGKK8FgPS
</commit_message>
<xml_diff>
--- a/social/marketing/menva-marketing-tracker.xlsx
+++ b/social/marketing/menva-marketing-tracker.xlsx
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>See it before you order it.</t>
+          <t>Real plate. Before you order it.</t>
         </is>
       </c>
       <c r="I2" s="6" t="n"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>The waiter's back. Still on page two.</t>
+          <t>Still on "jo bhi tum lo."</t>
         </is>
       </c>
       <c r="I3" s="6" t="n"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Friday, 9 pm. Pick one.</t>
+          <t>Nine pm. Pick one.</t>
         </is>
       </c>
       <c r="I5" s="6" t="n"/>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Group of eight. One order, not eight arguments.</t>
+          <t>One order. Not eight arguments.</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Your menu sells before anyone speaks.</t>
+          <t>Your quietest salesperson.</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>You ordered a starter. It arrived on a board.</t>
+          <t>You ordered a starter. It needed a chair.</t>
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Do I need an app?</t>
+          <t>Need an app?</t>
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Three things a menu line never tells you.</t>
+          <t>Three things your menu is hiding.</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Scariest thing in Lahore tonight? A menu with zero photos.</t>
+          <t>Scariest thing in Lahore tonight? Zero photos.</t>
         </is>
       </c>
       <c r="I21" s="6" t="n"/>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Outdoor plans just became indoor plans.</t>
+          <t>Indoor plans, effective immediately</t>
         </is>
       </c>
       <c r="I23" s="6" t="n"/>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Taste tests happen after you order. Sight tests happen before.</t>
+          <t>Taste tests happen after. Sight tests happen before.</t>
         </is>
       </c>
       <c r="I26" s="6" t="n"/>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Five signs your menu's costing you orders</t>
+          <t>Five signs your menu is working against you</t>
         </is>
       </c>
       <c r="I32" s="6" t="n"/>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>No AI-generated food. Not once, not ever.</t>
+          <t>No AI food. Not once. Not ever.</t>
         </is>
       </c>
       <c r="I34" s="6" t="n"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>"Is it worth the hype?"</t>
+          <t>The hype tax, itemised</t>
         </is>
       </c>
       <c r="I35" s="6" t="n"/>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>How the pilot works.</t>
+          <t>How the pilot actually works.</t>
         </is>
       </c>
       <c r="I37" s="6" t="n"/>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Let the menu do the describing. Let your team host.</t>
+          <t>Let the menu describe. Let your team host.</t>
         </is>
       </c>
       <c r="I42" s="6" t="n"/>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>Three myths about 3D menus.</t>
+          <t>Three myths, busted.</t>
         </is>
       </c>
       <c r="I47" s="6" t="n"/>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>Dinner for two became dinner for twelve.</t>
+          <t>Group of twelve, incoming</t>
         </is>
       </c>
       <c r="I53" s="6" t="n"/>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>Which Lahore restaurant should we scan next?</t>
+          <t>Restaurants on the list</t>
         </is>
       </c>
       <c r="I71" s="6" t="n"/>

</xml_diff>